<commit_message>
feature erweiterung fix2 final
</commit_message>
<xml_diff>
--- a/test_coverage_history.xlsx
+++ b/test_coverage_history.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
   <si>
     <t>Testlauf 1 - 2026-09-18 21:17:25</t>
   </si>
@@ -444,6 +444,102 @@
   </si>
   <si>
     <t>Testlauf 11 - 2026-09-26 21:55:45</t>
+  </si>
+  <si>
+    <t>Testlauf 12 - 2026-09-27 20:09:38</t>
+  </si>
+  <si>
+    <t>(377/457)</t>
+  </si>
+  <si>
+    <t>(1827/2792)</t>
+  </si>
+  <si>
+    <t>(7407/12453)</t>
+  </si>
+  <si>
+    <t>(3286/6255)</t>
+  </si>
+  <si>
+    <t>cli</t>
+  </si>
+  <si>
+    <t>(9/9)</t>
+  </si>
+  <si>
+    <t>(23/23)</t>
+  </si>
+  <si>
+    <t>(27/27)</t>
+  </si>
+  <si>
+    <t>(132/202)</t>
+  </si>
+  <si>
+    <t>(455/1228)</t>
+  </si>
+  <si>
+    <t>(2179/5531)</t>
+  </si>
+  <si>
+    <t>(779/2110)</t>
+  </si>
+  <si>
+    <t>(160/164)</t>
+  </si>
+  <si>
+    <t>(767/883)</t>
+  </si>
+  <si>
+    <t>(3067/4247)</t>
+  </si>
+  <si>
+    <t>(1466/2531)</t>
+  </si>
+  <si>
+    <t>(11/13)</t>
+  </si>
+  <si>
+    <t>(108/131)</t>
+  </si>
+  <si>
+    <t>(390/507)</t>
+  </si>
+  <si>
+    <t>(185/276)</t>
+  </si>
+  <si>
+    <t>(228/258)</t>
+  </si>
+  <si>
+    <t>(915/1097)</t>
+  </si>
+  <si>
+    <t>(472/737)</t>
+  </si>
+  <si>
+    <t>(8/8)</t>
+  </si>
+  <si>
+    <t>(28/31)</t>
+  </si>
+  <si>
+    <t>(115/160)</t>
+  </si>
+  <si>
+    <t>(22/54)</t>
+  </si>
+  <si>
+    <t>(88/102)</t>
+  </si>
+  <si>
+    <t>(290/407)</t>
+  </si>
+  <si>
+    <t>(161/286)</t>
+  </si>
+  <si>
+    <t>(0/22)</t>
   </si>
 </sst>
 </file>
@@ -489,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J184"/>
+  <dimension ref="A1:J202"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.0140705108643" customWidth="1"/>
@@ -4573,6 +4669,405 @@
         <v>65</v>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C189" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E189" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="G189" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="I189" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C190" s="0">
+        <v>0.82</v>
+      </c>
+      <c r="D190" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="E190" s="0">
+        <v>0.65</v>
+      </c>
+      <c r="F190" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="G190" s="0">
+        <v>0.59</v>
+      </c>
+      <c r="H190" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="I190" s="0">
+        <v>0.53</v>
+      </c>
+      <c r="J190" s="0" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C191" s="0">
+        <v>1</v>
+      </c>
+      <c r="D191" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E191" s="0">
+        <v>1</v>
+      </c>
+      <c r="F191" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G191" s="0">
+        <v>1</v>
+      </c>
+      <c r="H191" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="I191" s="0">
+        <v>1</v>
+      </c>
+      <c r="J191" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C192" s="0">
+        <v>1</v>
+      </c>
+      <c r="D192" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E192" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="F192" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="G192" s="0">
+        <v>0.84</v>
+      </c>
+      <c r="H192" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I192" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="J192" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C193" s="0">
+        <v>0.65</v>
+      </c>
+      <c r="D193" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="E193" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="F193" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="G193" s="0">
+        <v>0.39</v>
+      </c>
+      <c r="H193" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="I193" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="J193" s="0" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C194" s="0">
+        <v>1</v>
+      </c>
+      <c r="D194" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E194" s="0">
+        <v>1</v>
+      </c>
+      <c r="F194" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="G194" s="0">
+        <v>0.91</v>
+      </c>
+      <c r="H194" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="I194" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="J194" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C195" s="0">
+        <v>0.98</v>
+      </c>
+      <c r="D195" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="E195" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="F195" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="G195" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H195" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="I195" s="0">
+        <v>0.58</v>
+      </c>
+      <c r="J195" s="0" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C196" s="0">
+        <v>1</v>
+      </c>
+      <c r="D196" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E196" s="0">
+        <v>1</v>
+      </c>
+      <c r="F196" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G196" s="0">
+        <v>1</v>
+      </c>
+      <c r="H196" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I196" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="J196" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C197" s="0">
+        <v>0.85</v>
+      </c>
+      <c r="D197" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="E197" s="0">
+        <v>0.82</v>
+      </c>
+      <c r="F197" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="G197" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="H197" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="I197" s="0">
+        <v>0.67</v>
+      </c>
+      <c r="J197" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C198" s="0">
+        <v>0.97</v>
+      </c>
+      <c r="D198" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E198" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="F198" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="G198" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="H198" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="I198" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="J198" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C199" s="0">
+        <v>1</v>
+      </c>
+      <c r="D199" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E199" s="0">
+        <v>1</v>
+      </c>
+      <c r="F199" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="G199" s="0">
+        <v>1</v>
+      </c>
+      <c r="H199" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I199" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="J199" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C200" s="0">
+        <v>1</v>
+      </c>
+      <c r="D200" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="E200" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="F200" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="G200" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H200" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="I200" s="0">
+        <v>0.41</v>
+      </c>
+      <c r="J200" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C201" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="D201" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E201" s="0">
+        <v>0.86</v>
+      </c>
+      <c r="F201" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G201" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H201" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="I201" s="0">
+        <v>0.56</v>
+      </c>
+      <c r="J201" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C202" s="0">
+        <v>0</v>
+      </c>
+      <c r="D202" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="E202" s="0">
+        <v>0</v>
+      </c>
+      <c r="F202" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="G202" s="0">
+        <v>0</v>
+      </c>
+      <c r="H202" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="I202" s="0">
+        <v>0</v>
+      </c>
+      <c r="J202" s="0" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
kommentarfunktion bei coverage history
</commit_message>
<xml_diff>
--- a/test_coverage_history.xlsx
+++ b/test_coverage_history.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="193">
   <si>
     <t>Testlauf 1 - 2026-09-18 21:17:25</t>
   </si>
@@ -540,6 +540,57 @@
   </si>
   <si>
     <t>(0/22)</t>
+  </si>
+  <si>
+    <t>Testlauf 13 - 2026-10-01 13:24:52</t>
+  </si>
+  <si>
+    <t>(354/463)</t>
+  </si>
+  <si>
+    <t>(1725/2855)</t>
+  </si>
+  <si>
+    <t>(6931/12959)</t>
+  </si>
+  <si>
+    <t>(3160/6428)</t>
+  </si>
+  <si>
+    <t>(130/206)</t>
+  </si>
+  <si>
+    <t>(459/1248)</t>
+  </si>
+  <si>
+    <t>(2225/5635)</t>
+  </si>
+  <si>
+    <t>(799/2153)</t>
+  </si>
+  <si>
+    <t>(144/166)</t>
+  </si>
+  <si>
+    <t>(677/925)</t>
+  </si>
+  <si>
+    <t>(2627/4640)</t>
+  </si>
+  <si>
+    <t>(1336/2661)</t>
+  </si>
+  <si>
+    <t>(109/132)</t>
+  </si>
+  <si>
+    <t>(393/516)</t>
+  </si>
+  <si>
+    <t>(227/258)</t>
+  </si>
+  <si>
+    <t>(911/1097)</t>
   </si>
 </sst>
 </file>
@@ -585,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J202"/>
+  <dimension ref="A1:J220"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.0140705108643" customWidth="1"/>
@@ -5068,6 +5119,405 @@
         <v>63</v>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="0" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C207" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E207" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="G207" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="I207" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C208" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="D208" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="E208" s="0">
+        <v>0.6</v>
+      </c>
+      <c r="F208" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="G208" s="0">
+        <v>0.53</v>
+      </c>
+      <c r="H208" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="I208" s="0">
+        <v>0.49</v>
+      </c>
+      <c r="J208" s="0" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C209" s="0">
+        <v>1</v>
+      </c>
+      <c r="D209" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E209" s="0">
+        <v>1</v>
+      </c>
+      <c r="F209" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G209" s="0">
+        <v>1</v>
+      </c>
+      <c r="H209" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="I209" s="0">
+        <v>1</v>
+      </c>
+      <c r="J209" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C210" s="0">
+        <v>1</v>
+      </c>
+      <c r="D210" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E210" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="F210" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="G210" s="0">
+        <v>0.84</v>
+      </c>
+      <c r="H210" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I210" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="J210" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C211" s="0">
+        <v>0.63</v>
+      </c>
+      <c r="D211" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="E211" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="F211" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G211" s="0">
+        <v>0.39</v>
+      </c>
+      <c r="H211" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="I211" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="J211" s="0" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C212" s="0">
+        <v>1</v>
+      </c>
+      <c r="D212" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E212" s="0">
+        <v>1</v>
+      </c>
+      <c r="F212" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="G212" s="0">
+        <v>0.91</v>
+      </c>
+      <c r="H212" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="I212" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="J212" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C213" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="D213" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="E213" s="0">
+        <v>0.73</v>
+      </c>
+      <c r="F213" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="G213" s="0">
+        <v>0.57</v>
+      </c>
+      <c r="H213" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="I213" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="J213" s="0" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C214" s="0">
+        <v>1</v>
+      </c>
+      <c r="D214" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E214" s="0">
+        <v>1</v>
+      </c>
+      <c r="F214" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G214" s="0">
+        <v>1</v>
+      </c>
+      <c r="H214" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I214" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="J214" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C215" s="0">
+        <v>0.85</v>
+      </c>
+      <c r="D215" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="E215" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="F215" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="G215" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="H215" s="0" t="s">
+        <v>190</v>
+      </c>
+      <c r="I215" s="0">
+        <v>0.67</v>
+      </c>
+      <c r="J215" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C216" s="0">
+        <v>0.97</v>
+      </c>
+      <c r="D216" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E216" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="F216" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="G216" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="H216" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="I216" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="J216" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C217" s="0">
+        <v>1</v>
+      </c>
+      <c r="D217" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E217" s="0">
+        <v>1</v>
+      </c>
+      <c r="F217" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="G217" s="0">
+        <v>1</v>
+      </c>
+      <c r="H217" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I217" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="J217" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C218" s="0">
+        <v>0.38</v>
+      </c>
+      <c r="D218" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="E218" s="0">
+        <v>0.39</v>
+      </c>
+      <c r="F218" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="G218" s="0">
+        <v>0.21</v>
+      </c>
+      <c r="H218" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="I218" s="0">
+        <v>0.11</v>
+      </c>
+      <c r="J218" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C219" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="D219" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E219" s="0">
+        <v>0.86</v>
+      </c>
+      <c r="F219" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G219" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H219" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="I219" s="0">
+        <v>0.56</v>
+      </c>
+      <c r="J219" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C220" s="0">
+        <v>0</v>
+      </c>
+      <c r="D220" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="E220" s="0">
+        <v>0</v>
+      </c>
+      <c r="F220" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="G220" s="0">
+        <v>0</v>
+      </c>
+      <c r="H220" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="I220" s="0">
+        <v>0</v>
+      </c>
+      <c r="J220" s="0" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
vollständige umsetzung + fixes
</commit_message>
<xml_diff>
--- a/test_coverage_history.xlsx
+++ b/test_coverage_history.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
   <si>
     <t>Testlauf 1 - 2026-09-18 21:17:25</t>
   </si>
@@ -780,6 +780,21 @@
   </si>
   <si>
     <t>(3395/6428)</t>
+  </si>
+  <si>
+    <t>Testlauf 23 - 2026-10-01 23:22:23</t>
+  </si>
+  <si>
+    <t>Testlauf 24 - 2026-10-01 23:33:56</t>
+  </si>
+  <si>
+    <t>(385/463)</t>
+  </si>
+  <si>
+    <t>(1880/2860)</t>
+  </si>
+  <si>
+    <t>(7712/12976)</t>
   </si>
 </sst>
 </file>
@@ -825,7 +840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J382"/>
+  <dimension ref="A1:J418"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.0140705108643" customWidth="1"/>
@@ -9298,6 +9313,804 @@
         <v>244</v>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" s="0" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C387" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E387" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="G387" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="I387" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C388" s="0">
+        <v>0.82</v>
+      </c>
+      <c r="D388" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="E388" s="0">
+        <v>0.65</v>
+      </c>
+      <c r="F388" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="G388" s="0">
+        <v>0.59</v>
+      </c>
+      <c r="H388" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="I388" s="0">
+        <v>0.53</v>
+      </c>
+      <c r="J388" s="0" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C389" s="0">
+        <v>1</v>
+      </c>
+      <c r="D389" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E389" s="0">
+        <v>1</v>
+      </c>
+      <c r="F389" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G389" s="0">
+        <v>1</v>
+      </c>
+      <c r="H389" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="I389" s="0">
+        <v>1</v>
+      </c>
+      <c r="J389" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C390" s="0">
+        <v>1</v>
+      </c>
+      <c r="D390" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E390" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="F390" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="G390" s="0">
+        <v>0.84</v>
+      </c>
+      <c r="H390" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I390" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="J390" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C391" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="D391" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="E391" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="F391" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="G391" s="0">
+        <v>0.4</v>
+      </c>
+      <c r="H391" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="I391" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="J391" s="0" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C392" s="0">
+        <v>1</v>
+      </c>
+      <c r="D392" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E392" s="0">
+        <v>1</v>
+      </c>
+      <c r="F392" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="G392" s="0">
+        <v>0.91</v>
+      </c>
+      <c r="H392" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="I392" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="J392" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C393" s="0">
+        <v>0.98</v>
+      </c>
+      <c r="D393" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="E393" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="F393" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="G393" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H393" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="I393" s="0">
+        <v>0.58</v>
+      </c>
+      <c r="J393" s="0" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C394" s="0">
+        <v>1</v>
+      </c>
+      <c r="D394" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E394" s="0">
+        <v>1</v>
+      </c>
+      <c r="F394" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G394" s="0">
+        <v>1</v>
+      </c>
+      <c r="H394" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I394" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="J394" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C395" s="0">
+        <v>0.85</v>
+      </c>
+      <c r="D395" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="E395" s="0">
+        <v>0.81</v>
+      </c>
+      <c r="F395" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="G395" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="H395" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="I395" s="0">
+        <v>0.67</v>
+      </c>
+      <c r="J395" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C396" s="0">
+        <v>0.97</v>
+      </c>
+      <c r="D396" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E396" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="F396" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="G396" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="H396" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="I396" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="J396" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C397" s="0">
+        <v>1</v>
+      </c>
+      <c r="D397" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E397" s="0">
+        <v>1</v>
+      </c>
+      <c r="F397" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="G397" s="0">
+        <v>1</v>
+      </c>
+      <c r="H397" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I397" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="J397" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C398" s="0">
+        <v>1</v>
+      </c>
+      <c r="D398" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="E398" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="F398" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="G398" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H398" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="I398" s="0">
+        <v>0.41</v>
+      </c>
+      <c r="J398" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C399" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="D399" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E399" s="0">
+        <v>0.86</v>
+      </c>
+      <c r="F399" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G399" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H399" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="I399" s="0">
+        <v>0.56</v>
+      </c>
+      <c r="J399" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C400" s="0">
+        <v>1</v>
+      </c>
+      <c r="D400" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="E400" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="F400" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="G400" s="0">
+        <v>0.32</v>
+      </c>
+      <c r="H400" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="I400" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="J400" s="0" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="0" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C405" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E405" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="G405" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="I405" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C406" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="D406" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="E406" s="0">
+        <v>0.66</v>
+      </c>
+      <c r="F406" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="G406" s="0">
+        <v>0.59</v>
+      </c>
+      <c r="H406" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="I406" s="0">
+        <v>0.53</v>
+      </c>
+      <c r="J406" s="0" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C407" s="0">
+        <v>1</v>
+      </c>
+      <c r="D407" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E407" s="0">
+        <v>1</v>
+      </c>
+      <c r="F407" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G407" s="0">
+        <v>1</v>
+      </c>
+      <c r="H407" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="I407" s="0">
+        <v>1</v>
+      </c>
+      <c r="J407" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C408" s="0">
+        <v>1</v>
+      </c>
+      <c r="D408" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E408" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="F408" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="G408" s="0">
+        <v>0.84</v>
+      </c>
+      <c r="H408" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I408" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="J408" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C409" s="0">
+        <v>0.67</v>
+      </c>
+      <c r="D409" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="E409" s="0">
+        <v>0.38</v>
+      </c>
+      <c r="F409" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="G409" s="0">
+        <v>0.4</v>
+      </c>
+      <c r="H409" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="I409" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="J409" s="0" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C410" s="0">
+        <v>1</v>
+      </c>
+      <c r="D410" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E410" s="0">
+        <v>1</v>
+      </c>
+      <c r="F410" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="G410" s="0">
+        <v>0.91</v>
+      </c>
+      <c r="H410" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="I410" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="J410" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C411" s="0">
+        <v>0.98</v>
+      </c>
+      <c r="D411" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="E411" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="F411" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="G411" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H411" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="I411" s="0">
+        <v>0.58</v>
+      </c>
+      <c r="J411" s="0" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C412" s="0">
+        <v>1</v>
+      </c>
+      <c r="D412" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E412" s="0">
+        <v>1</v>
+      </c>
+      <c r="F412" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G412" s="0">
+        <v>1</v>
+      </c>
+      <c r="H412" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I412" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="J412" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C413" s="0">
+        <v>0.85</v>
+      </c>
+      <c r="D413" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="E413" s="0">
+        <v>0.81</v>
+      </c>
+      <c r="F413" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="G413" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="H413" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="I413" s="0">
+        <v>0.66</v>
+      </c>
+      <c r="J413" s="0" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C414" s="0">
+        <v>0.97</v>
+      </c>
+      <c r="D414" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E414" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="F414" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="G414" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="H414" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="I414" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="J414" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C415" s="0">
+        <v>1</v>
+      </c>
+      <c r="D415" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E415" s="0">
+        <v>1</v>
+      </c>
+      <c r="F415" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="G415" s="0">
+        <v>1</v>
+      </c>
+      <c r="H415" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I415" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="J415" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C416" s="0">
+        <v>1</v>
+      </c>
+      <c r="D416" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="E416" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="F416" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="G416" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H416" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="I416" s="0">
+        <v>0.41</v>
+      </c>
+      <c r="J416" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C417" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="D417" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E417" s="0">
+        <v>0.86</v>
+      </c>
+      <c r="F417" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G417" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H417" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="I417" s="0">
+        <v>0.56</v>
+      </c>
+      <c r="J417" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C418" s="0">
+        <v>1</v>
+      </c>
+      <c r="D418" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="E418" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="F418" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="G418" s="0">
+        <v>0.32</v>
+      </c>
+      <c r="H418" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="I418" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="J418" s="0" t="s">
+        <v>244</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>